<commit_message>
Bonding & Adventure Missions as Column G.
</commit_message>
<xml_diff>
--- a/research/breed-intelligence-database.xlsx
+++ b/research/breed-intelligence-database.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Breed Intelligence DB" sheetId="1" state="visible" r:id="rId1"/>
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Breed Groups Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="162913" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -2682,7 +2682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="13.44140625" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -2691,6 +2691,7 @@
     <col width="31.21875" customWidth="1" style="1" min="4" max="4"/>
     <col width="35.109375" customWidth="1" style="1" min="5" max="5"/>
     <col width="26.21875" customWidth="1" style="1" min="6" max="6"/>
+    <col width="31.21875" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2724,6 +2725,11 @@
           <t>Example Breeds</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Bonding &amp; Adventure Missions</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="57.6" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
@@ -2758,6 +2764,13 @@
           <t>Dachshund, Beagle, Shiba Inu, Italian Greyhound, Jack Russell Terrier</t>
         </is>
       </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>1. Explore a park or trail you've never visited together, letting the dog choose the direction at 3 intersections. (Adventure)
+2. Follow a scent trail laid with 5 hidden treats across a new outdoor space. (Adventure)
+3. Sit together outdoors after the walk and give calm praise while the dog decompresses. (Bonding)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="57.6" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
@@ -2792,6 +2805,13 @@
           <t>Poodle, Pembroke Welsh Corgi, German Shepherd, Border Collie, Australian Shepherd</t>
         </is>
       </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>1. Teach a new hand-signal command together, ending with a play reward. (Bonding)
+2. Play a 10-minute "find the toy" memory game indoors. (Bonding)
+3. Visit a new environment (cafe patio, new street) and practice calm focus amid novelty. (Adventure)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="57.6" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
@@ -2826,6 +2846,13 @@
           <t>Maltese, Pomeranian, Cavalier King Charles Spaniel, Bichon Frise, Golden Retriever, Cocker Spaniel, Samoyed</t>
         </is>
       </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>1. One-on-one cuddle/play session with their favorite person for 15 minutes. (Bonding)
+2. Supervised play date at home with a friend's dog. (Bonding)
+3. Group walk with another dog and owner to a new local spot. (Adventure)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="43.2" customHeight="1">
       <c r="A5" s="1" t="inlineStr">
@@ -2860,6 +2887,13 @@
           <t>Siberian Husky, Samoyed</t>
         </is>
       </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>1. Hike a new trail with elevation change for at least 30 minutes. (Adventure)
+2. Try a new outdoor activity together (paddleboard, beach run, open field). (Adventure)
+3. End the adventure with a relaxed shared rest stop, water break, and praise. (Bonding)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="57.6" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
@@ -2894,6 +2928,13 @@
           <t>French Bulldog, Shih Tzu, Italian Greyhound, Great Dane, Local Mixed Breed / Rescue, Tong Gau</t>
         </is>
       </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>1. Quiet 15-minute brushing/massage session on the couch. (Bonding)
+2. Sit together in a favorite calm spot (balcony, window seat) for 10 minutes of just being present. (Bonding)
+3. A slow, unhurried walk to one new-but-quiet nearby spot, no pressure to explore far. (Adventure)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="57.6" customHeight="1">
       <c r="A7" s="1" t="inlineStr">
@@ -2928,6 +2969,13 @@
           <t>Chihuahua, Yorkshire Terrier, Miniature Schnauzer, Doberman Pinscher, Rottweiler, Tong Gau</t>
         </is>
       </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>1. One-on-one structured training time with their primary person, ending in praise/play. (Bonding)
+2. Calm "watch duty" time together on the porch/balcony, rewarding relaxed alertness. (Bonding)
+3. Confidence-building walk to a new but controlled environment (quiet trail, empty lot). (Adventure)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="57.6" customHeight="1">
       <c r="A8" s="1" t="inlineStr">
@@ -2962,6 +3010,13 @@
           <t>Pug, Labrador Retriever, French Bulldog, Golden Retriever, Beagle</t>
         </is>
       </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>1. Hand-feed a portion of dinner during a bonding training session. (Bonding)
+2. Make a frozen treat or puzzle together and share the "unveiling" moment. (Bonding)
+3. Visit a new dog-friendly cafe or market for supervised, treat-motivated exploration. (Adventure)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="57.6" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
@@ -2994,6 +3049,13 @@
       <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Jack Russell Terrier, Poodle, Border Collie, Australian Shepherd, Siberian Husky</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>1. Timed fetch/sprint session at a new open space. (Adventure)
+2. Agility or obstacle circuit at a dog park or DIY backyard course. (Adventure)
+3. Post-workout cooldown stretch/massage together. (Bonding)</t>
         </is>
       </c>
     </row>

</xml_diff>